<commit_message>
Annotation & tidying code, hopefully final version of sorting code
</commit_message>
<xml_diff>
--- a/tetrode_data_JS.xlsx
+++ b/tetrode_data_JS.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="18">
   <si>
     <t xml:space="preserve">rat_ID</t>
   </si>
@@ -71,6 +71,12 @@
   </si>
   <si>
     <t xml:space="preserve">/home/isabella/Documents/isabella/jake/recording_data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">230124_r1299_t-maze_2_raw</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/home/isabella/Documents/isabella/jake/recording_data/r1299/2023-01-24</t>
   </si>
 </sst>
 </file>
@@ -131,7 +137,7 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
-      <family val="0"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -177,7 +183,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -195,6 +201,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -215,16 +225,17 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:O3"/>
   <sheetFormatPr defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12.63"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="21.39"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="26.53"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="26.39"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="7" style="0" width="12.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="16.94"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="8" style="0" width="12.63"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -280,13 +291,44 @@
         <v>64</v>
       </c>
       <c r="H2" s="4"/>
+      <c r="I2" s="5"/>
       <c r="J2" s="4"/>
-      <c r="K2" s="0" t="s">
+      <c r="K2" s="5" t="s">
         <v>14</v>
       </c>
       <c r="L2" s="4" t="s">
         <v>15</v>
       </c>
+      <c r="M2" s="5"/>
+      <c r="N2" s="5"/>
+      <c r="O2" s="5"/>
+    </row>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="5"/>
+      <c r="B3" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="5"/>
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G3" s="5" t="n">
+        <v>32</v>
+      </c>
+      <c r="H3" s="5"/>
+      <c r="I3" s="5"/>
+      <c r="J3" s="5"/>
+      <c r="K3" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="M3" s="5"/>
+      <c r="N3" s="5"/>
+      <c r="O3" s="5"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>